<commit_message>
Laboratorio 0 casi completo
</commit_message>
<xml_diff>
--- a/Unidad 1/G0_A2_estudiantes.xlsx
+++ b/Unidad 1/G0_A2_estudiantes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabian.sierra\Dropbox\Duoc\2025\SEGUNDO SEMESTRE\Creación Material\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Magol\Desktop\Inferencia estadistica\Unidad 1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48EF2C35-CD67-4E6B-9B8F-314CE6E6B224}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE5DDC8-604D-45B3-949C-5F989F804A94}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D2F66467-46D5-4128-A287-5FA9B7A5796A}"/>
+    <workbookView xWindow="1536" yWindow="1536" windowWidth="17280" windowHeight="8880" xr2:uid="{D2F66467-46D5-4128-A287-5FA9B7A5796A}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset_estudiantes" sheetId="1" r:id="rId1"/>
@@ -978,22 +978,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E902CEFB-7CEE-478E-B5A1-90C5380198B3}">
   <dimension ref="A1:J301"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.26953125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.6328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="13.7265625" style="1" customWidth="1"/>
-    <col min="11" max="16384" width="10.90625" style="2"/>
+    <col min="1" max="1" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.77734375" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="10.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1025,7 +1025,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>8</v>
       </c>
@@ -1057,7 +1057,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
@@ -1089,7 +1089,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1121,7 +1121,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>17</v>
       </c>
@@ -1153,7 +1153,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -1185,7 +1185,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
@@ -1217,7 +1217,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>15</v>
       </c>
@@ -1249,7 +1249,7 @@
         <v>2.6</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
@@ -1281,7 +1281,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
@@ -1313,7 +1313,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>16</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>17</v>
       </c>
@@ -1377,7 +1377,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>17</v>
       </c>
@@ -1409,7 +1409,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
@@ -1441,7 +1441,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -1505,7 +1505,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -1569,7 +1569,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>16</v>
       </c>
@@ -1601,7 +1601,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>16</v>
       </c>
@@ -1633,7 +1633,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>17</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>15</v>
       </c>
@@ -1729,7 +1729,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>8</v>
       </c>
@@ -1761,7 +1761,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>11</v>
       </c>
@@ -1793,7 +1793,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>8</v>
       </c>
@@ -1825,7 +1825,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -1857,7 +1857,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>16</v>
       </c>
@@ -1889,7 +1889,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>16</v>
       </c>
@@ -1921,7 +1921,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>17</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>15</v>
       </c>
@@ -1985,7 +1985,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>11</v>
       </c>
@@ -2017,7 +2017,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>11</v>
       </c>
@@ -2049,7 +2049,7 @@
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>11</v>
       </c>
@@ -2081,7 +2081,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>17</v>
       </c>
@@ -2113,7 +2113,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>15</v>
       </c>
@@ -2145,7 +2145,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>8</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>17</v>
       </c>
@@ -2209,7 +2209,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>11</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>16</v>
       </c>
@@ -2273,7 +2273,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>15</v>
       </c>
@@ -2305,7 +2305,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>8</v>
       </c>
@@ -2337,7 +2337,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>16</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>15</v>
       </c>
@@ -2401,7 +2401,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>8</v>
       </c>
@@ -2433,7 +2433,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>8</v>
       </c>
@@ -2465,7 +2465,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>8</v>
       </c>
@@ -2497,7 +2497,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>8</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>11</v>
       </c>
@@ -2561,7 +2561,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>15</v>
       </c>
@@ -2593,7 +2593,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>15</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
@@ -2657,7 +2657,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>11</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>15</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>8</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>16</v>
       </c>
@@ -2785,7 +2785,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>11</v>
       </c>
@@ -2817,7 +2817,7 @@
         <v>6.1</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>15</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>17</v>
       </c>
@@ -2881,7 +2881,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>15</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>8</v>
       </c>
@@ -2945,7 +2945,7 @@
         <v>6.1</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>17</v>
       </c>
@@ -2977,7 +2977,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>8</v>
       </c>
@@ -3009,7 +3009,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>11</v>
       </c>
@@ -3041,7 +3041,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>16</v>
       </c>
@@ -3073,7 +3073,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>17</v>
       </c>
@@ -3105,7 +3105,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>11</v>
       </c>
@@ -3137,7 +3137,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="68" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>8</v>
       </c>
@@ -3169,7 +3169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>17</v>
       </c>
@@ -3201,7 +3201,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="70" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>17</v>
       </c>
@@ -3233,7 +3233,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>15</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="72" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>11</v>
       </c>
@@ -3297,7 +3297,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="73" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>17</v>
       </c>
@@ -3329,7 +3329,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>16</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="75" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>16</v>
       </c>
@@ -3393,7 +3393,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="76" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>15</v>
       </c>
@@ -3425,7 +3425,7 @@
         <v>2.9</v>
       </c>
     </row>
-    <row r="77" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>17</v>
       </c>
@@ -3457,7 +3457,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>15</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="79" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>15</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>15</v>
       </c>
@@ -3553,7 +3553,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>17</v>
       </c>
@@ -3585,7 +3585,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>17</v>
       </c>
@@ -3617,7 +3617,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>8</v>
       </c>
@@ -3649,7 +3649,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>15</v>
       </c>
@@ -3681,7 +3681,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>15</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>15</v>
       </c>
@@ -3745,7 +3745,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>15</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>16</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>17</v>
       </c>
@@ -3841,7 +3841,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>15</v>
       </c>
@@ -3873,7 +3873,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>17</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>11</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>15</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>17</v>
       </c>
@@ -4001,7 +4001,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>8</v>
       </c>
@@ -4033,7 +4033,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>15</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="97" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>11</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>15</v>
       </c>
@@ -4129,7 +4129,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>17</v>
       </c>
@@ -4161,7 +4161,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="100" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>16</v>
       </c>
@@ -4193,7 +4193,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>16</v>
       </c>
@@ -4225,7 +4225,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>15</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="103" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>16</v>
       </c>
@@ -4289,7 +4289,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>17</v>
       </c>
@@ -4321,7 +4321,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>17</v>
       </c>
@@ -4353,7 +4353,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>16</v>
       </c>
@@ -4385,7 +4385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>15</v>
       </c>
@@ -4417,7 +4417,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>17</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="109" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>15</v>
       </c>
@@ -4481,7 +4481,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>11</v>
       </c>
@@ -4513,7 +4513,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="111" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>11</v>
       </c>
@@ -4545,7 +4545,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>17</v>
       </c>
@@ -4577,7 +4577,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>11</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>11</v>
       </c>
@@ -4641,7 +4641,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>15</v>
       </c>
@@ -4673,7 +4673,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>11</v>
       </c>
@@ -4705,7 +4705,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>15</v>
       </c>
@@ -4737,7 +4737,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>16</v>
       </c>
@@ -4769,7 +4769,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>11</v>
       </c>
@@ -4801,7 +4801,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>11</v>
       </c>
@@ -4833,7 +4833,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>11</v>
       </c>
@@ -4865,7 +4865,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>11</v>
       </c>
@@ -4897,7 +4897,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>16</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>16</v>
       </c>
@@ -4961,7 +4961,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>17</v>
       </c>
@@ -4993,7 +4993,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>16</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>16</v>
       </c>
@@ -5057,7 +5057,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>11</v>
       </c>
@@ -5089,7 +5089,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="129" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>8</v>
       </c>
@@ -5121,7 +5121,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="130" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>8</v>
       </c>
@@ -5153,7 +5153,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="131" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>16</v>
       </c>
@@ -5185,7 +5185,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="132" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>17</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>16</v>
       </c>
@@ -5249,7 +5249,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="134" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>8</v>
       </c>
@@ -5281,7 +5281,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="135" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>11</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="136" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>11</v>
       </c>
@@ -5345,7 +5345,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="137" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>17</v>
       </c>
@@ -5377,7 +5377,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="138" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>8</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="139" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>15</v>
       </c>
@@ -5441,7 +5441,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="140" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>17</v>
       </c>
@@ -5473,7 +5473,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="141" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>11</v>
       </c>
@@ -5505,7 +5505,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="142" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>15</v>
       </c>
@@ -5537,7 +5537,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="143" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>17</v>
       </c>
@@ -5569,7 +5569,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="144" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>17</v>
       </c>
@@ -5601,7 +5601,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>16</v>
       </c>
@@ -5633,7 +5633,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>17</v>
       </c>
@@ -5665,7 +5665,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>15</v>
       </c>
@@ -5697,7 +5697,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>17</v>
       </c>
@@ -5729,7 +5729,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>16</v>
       </c>
@@ -5761,7 +5761,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>17</v>
       </c>
@@ -5793,7 +5793,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>8</v>
       </c>
@@ -5825,7 +5825,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>8</v>
       </c>
@@ -5857,7 +5857,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>8</v>
       </c>
@@ -5889,7 +5889,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>17</v>
       </c>
@@ -5921,7 +5921,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>15</v>
       </c>
@@ -5953,7 +5953,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>8</v>
       </c>
@@ -5985,7 +5985,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>15</v>
       </c>
@@ -6017,7 +6017,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>17</v>
       </c>
@@ -6049,7 +6049,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>17</v>
       </c>
@@ -6081,7 +6081,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>15</v>
       </c>
@@ -6113,7 +6113,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="161" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>15</v>
       </c>
@@ -6145,7 +6145,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="162" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>8</v>
       </c>
@@ -6177,7 +6177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="163" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>11</v>
       </c>
@@ -6209,7 +6209,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="164" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>16</v>
       </c>
@@ -6241,7 +6241,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="165" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>15</v>
       </c>
@@ -6273,7 +6273,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="166" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>8</v>
       </c>
@@ -6305,7 +6305,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="167" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A167" s="1" t="s">
         <v>15</v>
       </c>
@@ -6337,7 +6337,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="168" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A168" s="1" t="s">
         <v>8</v>
       </c>
@@ -6369,7 +6369,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="169" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A169" s="1" t="s">
         <v>8</v>
       </c>
@@ -6401,7 +6401,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="170" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A170" s="1" t="s">
         <v>15</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="171" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A171" s="1" t="s">
         <v>17</v>
       </c>
@@ -6465,7 +6465,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="172" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A172" s="1" t="s">
         <v>15</v>
       </c>
@@ -6497,7 +6497,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="173" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A173" s="1" t="s">
         <v>17</v>
       </c>
@@ -6529,7 +6529,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="174" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A174" s="1" t="s">
         <v>15</v>
       </c>
@@ -6561,7 +6561,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="175" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A175" s="1" t="s">
         <v>15</v>
       </c>
@@ -6593,7 +6593,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="176" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A176" s="1" t="s">
         <v>15</v>
       </c>
@@ -6625,7 +6625,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="177" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A177" s="1" t="s">
         <v>15</v>
       </c>
@@ -6657,7 +6657,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="178" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A178" s="1" t="s">
         <v>16</v>
       </c>
@@ -6689,7 +6689,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="179" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A179" s="1" t="s">
         <v>16</v>
       </c>
@@ -6721,7 +6721,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="180" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A180" s="1" t="s">
         <v>11</v>
       </c>
@@ -6753,7 +6753,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="181" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A181" s="1" t="s">
         <v>11</v>
       </c>
@@ -6785,7 +6785,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="182" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A182" s="1" t="s">
         <v>16</v>
       </c>
@@ -6817,7 +6817,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="183" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A183" s="1" t="s">
         <v>16</v>
       </c>
@@ -6849,7 +6849,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="184" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A184" s="1" t="s">
         <v>11</v>
       </c>
@@ -6881,7 +6881,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="185" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A185" s="1" t="s">
         <v>17</v>
       </c>
@@ -6913,7 +6913,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="186" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A186" s="1" t="s">
         <v>8</v>
       </c>
@@ -6945,7 +6945,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="187" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A187" s="1" t="s">
         <v>17</v>
       </c>
@@ -6977,7 +6977,7 @@
         <v>2.4</v>
       </c>
     </row>
-    <row r="188" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A188" s="1" t="s">
         <v>11</v>
       </c>
@@ -7009,7 +7009,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="189" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="189" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A189" s="1" t="s">
         <v>17</v>
       </c>
@@ -7041,7 +7041,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="190" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="190" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A190" s="1" t="s">
         <v>15</v>
       </c>
@@ -7073,7 +7073,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="191" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="191" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A191" s="1" t="s">
         <v>11</v>
       </c>
@@ -7105,7 +7105,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="192" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A192" s="1" t="s">
         <v>8</v>
       </c>
@@ -7137,7 +7137,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="193" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A193" s="1" t="s">
         <v>8</v>
       </c>
@@ -7169,7 +7169,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="194" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A194" s="1" t="s">
         <v>11</v>
       </c>
@@ -7201,7 +7201,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="195" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A195" s="1" t="s">
         <v>15</v>
       </c>
@@ -7233,7 +7233,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="196" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A196" s="1" t="s">
         <v>16</v>
       </c>
@@ -7265,7 +7265,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="197" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="197" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A197" s="1" t="s">
         <v>15</v>
       </c>
@@ -7297,7 +7297,7 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="198" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A198" s="1" t="s">
         <v>15</v>
       </c>
@@ -7329,7 +7329,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="199" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A199" s="1" t="s">
         <v>8</v>
       </c>
@@ -7361,7 +7361,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="200" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A200" s="1" t="s">
         <v>17</v>
       </c>
@@ -7393,7 +7393,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="201" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A201" s="1" t="s">
         <v>17</v>
       </c>
@@ -7425,7 +7425,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="202" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A202" s="1" t="s">
         <v>17</v>
       </c>
@@ -7457,7 +7457,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="203" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A203" s="1" t="s">
         <v>8</v>
       </c>
@@ -7489,7 +7489,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A204" s="1" t="s">
         <v>8</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="205" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A205" s="1" t="s">
         <v>8</v>
       </c>
@@ -7553,7 +7553,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="206" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A206" s="1" t="s">
         <v>16</v>
       </c>
@@ -7585,7 +7585,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="207" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A207" s="1" t="s">
         <v>16</v>
       </c>
@@ -7617,7 +7617,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="208" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A208" s="1" t="s">
         <v>17</v>
       </c>
@@ -7649,7 +7649,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="209" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="209" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A209" s="1" t="s">
         <v>15</v>
       </c>
@@ -7681,7 +7681,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="210" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="210" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A210" s="1" t="s">
         <v>15</v>
       </c>
@@ -7713,7 +7713,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="211" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="211" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A211" s="1" t="s">
         <v>15</v>
       </c>
@@ -7745,7 +7745,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="212" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="212" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A212" s="1" t="s">
         <v>17</v>
       </c>
@@ -7777,7 +7777,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="213" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="213" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A213" s="1" t="s">
         <v>15</v>
       </c>
@@ -7809,7 +7809,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="214" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="214" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A214" s="1" t="s">
         <v>17</v>
       </c>
@@ -7841,7 +7841,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="215" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="215" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A215" s="1" t="s">
         <v>8</v>
       </c>
@@ -7873,7 +7873,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="216" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="216" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A216" s="1" t="s">
         <v>11</v>
       </c>
@@ -7905,7 +7905,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="217" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="217" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A217" s="1" t="s">
         <v>17</v>
       </c>
@@ -7937,7 +7937,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="218" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="218" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A218" s="1" t="s">
         <v>16</v>
       </c>
@@ -7969,7 +7969,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="219" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="219" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A219" s="1" t="s">
         <v>17</v>
       </c>
@@ -8001,7 +8001,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="220" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="220" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A220" s="1" t="s">
         <v>11</v>
       </c>
@@ -8033,7 +8033,7 @@
         <v>4.2</v>
       </c>
     </row>
-    <row r="221" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="221" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A221" s="1" t="s">
         <v>8</v>
       </c>
@@ -8065,7 +8065,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="222" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="222" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A222" s="1" t="s">
         <v>16</v>
       </c>
@@ -8097,7 +8097,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="223" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="223" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A223" s="1" t="s">
         <v>17</v>
       </c>
@@ -8129,7 +8129,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="224" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="224" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A224" s="1" t="s">
         <v>8</v>
       </c>
@@ -8161,7 +8161,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="225" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="225" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A225" s="1" t="s">
         <v>11</v>
       </c>
@@ -8193,7 +8193,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="226" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="226" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A226" s="1" t="s">
         <v>11</v>
       </c>
@@ -8225,7 +8225,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="227" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="227" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A227" s="1" t="s">
         <v>11</v>
       </c>
@@ -8257,7 +8257,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="228" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="228" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A228" s="1" t="s">
         <v>15</v>
       </c>
@@ -8289,7 +8289,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="229" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="229" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A229" s="1" t="s">
         <v>15</v>
       </c>
@@ -8321,7 +8321,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="230" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A230" s="1" t="s">
         <v>17</v>
       </c>
@@ -8353,7 +8353,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="231" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A231" s="1" t="s">
         <v>11</v>
       </c>
@@ -8385,7 +8385,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="232" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="232" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A232" s="1" t="s">
         <v>16</v>
       </c>
@@ -8417,7 +8417,7 @@
         <v>3.4</v>
       </c>
     </row>
-    <row r="233" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="233" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A233" s="1" t="s">
         <v>11</v>
       </c>
@@ -8449,7 +8449,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="234" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="234" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A234" s="1" t="s">
         <v>16</v>
       </c>
@@ -8481,7 +8481,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="235" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="235" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A235" s="1" t="s">
         <v>16</v>
       </c>
@@ -8513,7 +8513,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="236" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="236" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A236" s="1" t="s">
         <v>16</v>
       </c>
@@ -8545,7 +8545,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="237" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A237" s="1" t="s">
         <v>17</v>
       </c>
@@ -8577,7 +8577,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="238" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A238" s="1" t="s">
         <v>16</v>
       </c>
@@ -8609,7 +8609,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="239" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="239" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A239" s="1" t="s">
         <v>11</v>
       </c>
@@ -8641,7 +8641,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="240" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="240" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A240" s="1" t="s">
         <v>15</v>
       </c>
@@ -8673,7 +8673,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="241" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="241" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A241" s="1" t="s">
         <v>8</v>
       </c>
@@ -8705,7 +8705,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="242" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="242" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A242" s="1" t="s">
         <v>11</v>
       </c>
@@ -8737,7 +8737,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="243" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="243" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A243" s="1" t="s">
         <v>16</v>
       </c>
@@ -8769,7 +8769,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="244" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="244" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A244" s="1" t="s">
         <v>17</v>
       </c>
@@ -8801,7 +8801,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="245" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="245" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A245" s="1" t="s">
         <v>8</v>
       </c>
@@ -8833,7 +8833,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="246" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="246" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A246" s="1" t="s">
         <v>8</v>
       </c>
@@ -8865,7 +8865,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="247" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="247" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A247" s="1" t="s">
         <v>8</v>
       </c>
@@ -8897,7 +8897,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="248" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="248" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A248" s="1" t="s">
         <v>8</v>
       </c>
@@ -8929,7 +8929,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="249" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="249" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A249" s="1" t="s">
         <v>15</v>
       </c>
@@ -8961,7 +8961,7 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="250" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="250" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A250" s="1" t="s">
         <v>8</v>
       </c>
@@ -8993,7 +8993,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="251" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="251" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A251" s="1" t="s">
         <v>17</v>
       </c>
@@ -9025,7 +9025,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="252" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="252" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A252" s="1" t="s">
         <v>16</v>
       </c>
@@ -9057,7 +9057,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="253" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="253" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A253" s="1" t="s">
         <v>11</v>
       </c>
@@ -9089,7 +9089,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="254" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="254" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A254" s="1" t="s">
         <v>17</v>
       </c>
@@ -9121,7 +9121,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="255" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="255" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A255" s="1" t="s">
         <v>17</v>
       </c>
@@ -9153,7 +9153,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="256" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="256" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A256" s="1" t="s">
         <v>8</v>
       </c>
@@ -9185,7 +9185,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="257" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="257" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A257" s="1" t="s">
         <v>16</v>
       </c>
@@ -9217,7 +9217,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="258" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="258" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A258" s="1" t="s">
         <v>15</v>
       </c>
@@ -9249,7 +9249,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="259" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="259" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A259" s="1" t="s">
         <v>17</v>
       </c>
@@ -9281,7 +9281,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="260" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="260" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A260" s="1" t="s">
         <v>15</v>
       </c>
@@ -9313,7 +9313,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="261" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="261" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A261" s="1" t="s">
         <v>15</v>
       </c>
@@ -9345,7 +9345,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="262" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="262" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A262" s="1" t="s">
         <v>15</v>
       </c>
@@ -9377,7 +9377,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="263" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="263" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A263" s="1" t="s">
         <v>17</v>
       </c>
@@ -9409,7 +9409,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="264" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="264" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A264" s="1" t="s">
         <v>17</v>
       </c>
@@ -9441,7 +9441,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="265" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="265" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A265" s="1" t="s">
         <v>17</v>
       </c>
@@ -9473,7 +9473,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="266" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="266" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A266" s="1" t="s">
         <v>15</v>
       </c>
@@ -9505,7 +9505,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="267" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A267" s="1" t="s">
         <v>17</v>
       </c>
@@ -9537,7 +9537,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="268" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A268" s="1" t="s">
         <v>17</v>
       </c>
@@ -9569,7 +9569,7 @@
         <v>5.6</v>
       </c>
     </row>
-    <row r="269" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A269" s="1" t="s">
         <v>8</v>
       </c>
@@ -9601,7 +9601,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="270" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A270" s="1" t="s">
         <v>17</v>
       </c>
@@ -9633,7 +9633,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="271" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A271" s="1" t="s">
         <v>16</v>
       </c>
@@ -9665,7 +9665,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="272" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A272" s="1" t="s">
         <v>16</v>
       </c>
@@ -9697,7 +9697,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="273" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A273" s="1" t="s">
         <v>11</v>
       </c>
@@ -9729,7 +9729,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="274" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A274" s="1" t="s">
         <v>8</v>
       </c>
@@ -9761,7 +9761,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="275" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A275" s="1" t="s">
         <v>15</v>
       </c>
@@ -9793,7 +9793,7 @@
         <v>4.4000000000000004</v>
       </c>
     </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="276" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A276" s="1" t="s">
         <v>16</v>
       </c>
@@ -9825,7 +9825,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="277" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A277" s="1" t="s">
         <v>11</v>
       </c>
@@ -9857,7 +9857,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="278" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A278" s="1" t="s">
         <v>8</v>
       </c>
@@ -9889,7 +9889,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="279" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A279" s="1" t="s">
         <v>8</v>
       </c>
@@ -9921,7 +9921,7 @@
         <v>3.6</v>
       </c>
     </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="280" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A280" s="1" t="s">
         <v>17</v>
       </c>
@@ -9953,7 +9953,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="281" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A281" s="1" t="s">
         <v>16</v>
       </c>
@@ -9985,7 +9985,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="282" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A282" s="1" t="s">
         <v>16</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="283" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A283" s="1" t="s">
         <v>8</v>
       </c>
@@ -10049,7 +10049,7 @@
         <v>3.8</v>
       </c>
     </row>
-    <row r="284" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="284" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A284" s="1" t="s">
         <v>11</v>
       </c>
@@ -10081,7 +10081,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="285" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="285" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A285" s="1" t="s">
         <v>17</v>
       </c>
@@ -10113,7 +10113,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="286" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="286" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A286" s="1" t="s">
         <v>17</v>
       </c>
@@ -10145,7 +10145,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="287" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="287" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A287" s="1" t="s">
         <v>15</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>4.3</v>
       </c>
     </row>
-    <row r="288" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="288" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A288" s="1" t="s">
         <v>8</v>
       </c>
@@ -10209,7 +10209,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="289" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="289" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A289" s="1" t="s">
         <v>11</v>
       </c>
@@ -10241,7 +10241,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="290" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="290" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A290" s="1" t="s">
         <v>8</v>
       </c>
@@ -10273,7 +10273,7 @@
         <v>3.7</v>
       </c>
     </row>
-    <row r="291" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="291" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A291" s="1" t="s">
         <v>17</v>
       </c>
@@ -10305,7 +10305,7 @@
         <v>5.3</v>
       </c>
     </row>
-    <row r="292" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="292" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A292" s="1" t="s">
         <v>16</v>
       </c>
@@ -10337,7 +10337,7 @@
         <v>3.9</v>
       </c>
     </row>
-    <row r="293" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="293" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A293" s="1" t="s">
         <v>15</v>
       </c>
@@ -10369,7 +10369,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="294" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="294" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A294" s="1" t="s">
         <v>17</v>
       </c>
@@ -10401,7 +10401,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="295" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="295" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A295" s="1" t="s">
         <v>15</v>
       </c>
@@ -10433,7 +10433,7 @@
         <v>4.0999999999999996</v>
       </c>
     </row>
-    <row r="296" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="296" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A296" s="1" t="s">
         <v>16</v>
       </c>
@@ -10465,7 +10465,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="297" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="297" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A297" s="1" t="s">
         <v>16</v>
       </c>
@@ -10497,7 +10497,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="298" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="298" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A298" s="1" t="s">
         <v>17</v>
       </c>
@@ -10529,7 +10529,7 @@
         <v>6.9</v>
       </c>
     </row>
-    <row r="299" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="299" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A299" s="1" t="s">
         <v>11</v>
       </c>
@@ -10561,7 +10561,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="300" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="300" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A300" s="1" t="s">
         <v>15</v>
       </c>
@@ -10593,7 +10593,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="301" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="301" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A301" s="1" t="s">
         <v>8</v>
       </c>
@@ -10631,6 +10631,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x01010053980EFE0110084CBF3D893419E7BBE7" ma:contentTypeVersion="20" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="db9aaa4c57baa6b209dc8c64ff0e582a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="0a0d3458-2d9d-4ad2-ba24-97c7ba1c7dce" xmlns:ns3="64124649-a104-4bf2-a02a-5e406def83d9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="587f8181b8924f162aa46c928d78e6b3" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -10902,15 +10911,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -10925,13 +10925,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E9329A-33D5-4C76-9232-079E9164050A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B73A195-43EF-4F7A-81D3-37B42542CE5B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B73A195-43EF-4F7A-81D3-37B42542CE5B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{42E9329A-33D5-4C76-9232-079E9164050A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="0a0d3458-2d9d-4ad2-ba24-97c7ba1c7dce"/>
+    <ds:schemaRef ds:uri="64124649-a104-4bf2-a02a-5e406def83d9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997F6A8E-3C4D-43FD-903F-18E3F7B7EF20}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{997F6A8E-3C4D-43FD-903F-18E3F7B7EF20}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="64124649-a104-4bf2-a02a-5e406def83d9"/>
+    <ds:schemaRef ds:uri="0a0d3458-2d9d-4ad2-ba24-97c7ba1c7dce"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>